<commit_message>
Update daily stock valuation report
</commit_message>
<xml_diff>
--- a/data/pe_valuation_history.xlsx
+++ b/data/pe_valuation_history.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS10"/>
+  <dimension ref="A1:AS19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -892,7 +892,7 @@
         <v>226.549723637419</v>
       </c>
       <c r="AB3" t="n">
-        <v>490.6936524638191</v>
+        <v>490.6936524638192</v>
       </c>
       <c r="AC3" t="n">
         <v>124</v>
@@ -922,7 +922,7 @@
         <v>1.745635268477249</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.9354838709677419</v>
+        <v>0.935483870967742</v>
       </c>
       <c r="AM3" t="n">
         <v>214.728675813495</v>
@@ -1019,7 +1019,7 @@
         <v>34.92747542249608</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.00881231720520243</v>
+        <v>-0.0088123172052024</v>
       </c>
       <c r="U4" t="n">
         <v>0.4603174603174603</v>
@@ -1070,7 +1070,7 @@
         <v>34.70906596802268</v>
       </c>
       <c r="AK4" t="n">
-        <v>-0.02194268614028044</v>
+        <v>-0.0219426861402804</v>
       </c>
       <c r="AL4" t="n">
         <v>0.4274193548387097</v>
@@ -1152,7 +1152,7 @@
         <v>57.19493248774063</v>
       </c>
       <c r="N5" t="n">
-        <v>93.87329577470153</v>
+        <v>93.87329577470152</v>
       </c>
       <c r="O5" t="n">
         <v>74.91719886917585</v>
@@ -1161,7 +1161,7 @@
         <v>78.39571411846676</v>
       </c>
       <c r="Q5" t="n">
-        <v>9.711013572373497</v>
+        <v>9.711013572373496</v>
       </c>
       <c r="R5" t="n">
         <v>61.29707440530581</v>
@@ -1173,7 +1173,7 @@
         <v>-1.116510525741735</v>
       </c>
       <c r="U5" t="n">
-        <v>0.253968253968254</v>
+        <v>0.2539682539682539</v>
       </c>
       <c r="V5" t="n">
         <v>344.3134935761985</v>
@@ -1203,7 +1203,7 @@
         <v>57.19493248774063</v>
       </c>
       <c r="AE5" t="n">
-        <v>93.87329577470153</v>
+        <v>93.87329577470152</v>
       </c>
       <c r="AF5" t="n">
         <v>72.7265189141975</v>
@@ -1324,7 +1324,7 @@
         <v>-0.6813979368487536</v>
       </c>
       <c r="U6" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.238095238095238</v>
       </c>
       <c r="V6" t="n">
         <v>330.7495644540284</v>
@@ -1366,7 +1366,7 @@
         <v>1.920880039883152</v>
       </c>
       <c r="AI6" t="n">
-        <v>27.64653123825595</v>
+        <v>27.64653123825596</v>
       </c>
       <c r="AJ6" t="n">
         <v>32.6446195792587</v>
@@ -1375,7 +1375,7 @@
         <v>-1.014415354377868</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.1370967741935484</v>
+        <v>0.1370967741935483</v>
       </c>
       <c r="AM6" t="n">
         <v>330.7495644540284</v>
@@ -1460,7 +1460,7 @@
         <v>24.81354057111685</v>
       </c>
       <c r="P7" t="n">
-        <v>24.45551391965331</v>
+        <v>24.4555139196533</v>
       </c>
       <c r="Q7" t="n">
         <v>2.599953635337401</v>
@@ -1623,7 +1623,7 @@
         <v>26.50944369222463</v>
       </c>
       <c r="T8" t="n">
-        <v>0.03203632796460248</v>
+        <v>0.0320363279646024</v>
       </c>
       <c r="U8" t="n">
         <v>0.5238095238095238</v>
@@ -1641,7 +1641,7 @@
         <v>396.1754903124479</v>
       </c>
       <c r="Z8" t="n">
-        <v>435.8921394113643</v>
+        <v>435.8921394113642</v>
       </c>
       <c r="AA8" t="n">
         <v>389.6339176600243</v>
@@ -1662,7 +1662,7 @@
         <v>27.43189715615672</v>
       </c>
       <c r="AG8" t="n">
-        <v>25.35834965517999</v>
+        <v>25.35834965518</v>
       </c>
       <c r="AH8" t="n">
         <v>4.118216138579381</v>
@@ -1759,13 +1759,13 @@
         <v>42.60474344487245</v>
       </c>
       <c r="O9" t="n">
-        <v>38.41600789652239</v>
+        <v>38.4160078965224</v>
       </c>
       <c r="P9" t="n">
         <v>37.71936770955563</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.917248392190739</v>
+        <v>1.917248392190738</v>
       </c>
       <c r="R9" t="n">
         <v>36.41976247191899</v>
@@ -1789,7 +1789,7 @@
         <v>119.0896244792194</v>
       </c>
       <c r="Y9" t="n">
-        <v>113.1461544634281</v>
+        <v>113.1461544634282</v>
       </c>
       <c r="Z9" t="n">
         <v>125.0330944950107</v>
@@ -1804,13 +1804,13 @@
         <v>89</v>
       </c>
       <c r="AD9" t="n">
-        <v>3.489557264641911</v>
+        <v>3.48955726464191</v>
       </c>
       <c r="AE9" t="n">
         <v>42.60474344487245</v>
       </c>
       <c r="AF9" t="n">
-        <v>24.66089290957747</v>
+        <v>24.66089290957746</v>
       </c>
       <c r="AG9" t="n">
         <v>32.4901173708467</v>
@@ -1825,10 +1825,10 @@
         <v>39.10988125405291</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.1186763619131203</v>
+        <v>0.1186763619131202</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.3483146067415731</v>
+        <v>0.348314606741573</v>
       </c>
       <c r="AM9" t="n">
         <v>10.81762752038992</v>
@@ -1928,7 +1928,7 @@
         <v>-1.672769915643793</v>
       </c>
       <c r="U10" t="n">
-        <v>0.01587301587301587</v>
+        <v>0.0158730158730158</v>
       </c>
       <c r="V10" t="n">
         <v>204.7859172733417</v>
@@ -1961,7 +1961,7 @@
         <v>48.11020520268654</v>
       </c>
       <c r="AF10" t="n">
-        <v>38.32041307606467</v>
+        <v>38.32041307606468</v>
       </c>
       <c r="AG10" t="n">
         <v>37.37551007952008</v>
@@ -1979,7 +1979,7 @@
         <v>-1.731914848513478</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.01408450704225352</v>
+        <v>0.0140845070422535</v>
       </c>
       <c r="AM10" t="n">
         <v>204.7859172733417</v>
@@ -2001,6 +2001,1365 @@
       </c>
       <c r="AS10" t="n">
         <v>288.2239191794881</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>301.54</v>
+      </c>
+      <c r="I11" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="J11" t="n">
+        <v>36.506054</v>
+      </c>
+      <c r="K11" t="n">
+        <v>67</v>
+      </c>
+      <c r="L11" t="n">
+        <v>62</v>
+      </c>
+      <c r="M11" t="n">
+        <v>31.21898795984968</v>
+      </c>
+      <c r="N11" t="n">
+        <v>38.15980777324834</v>
+      </c>
+      <c r="O11" t="n">
+        <v>34.29914316528635</v>
+      </c>
+      <c r="P11" t="n">
+        <v>34.20253319076345</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>2.086475296404038</v>
+      </c>
+      <c r="R11" t="n">
+        <v>31.83607656744462</v>
+      </c>
+      <c r="S11" t="n">
+        <v>37.38147763305368</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1.057722005392147</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.7903225806451613</v>
+      </c>
+      <c r="V11" t="n">
+        <v>257.8688405483584</v>
+      </c>
+      <c r="W11" t="n">
+        <v>315.2000122070312</v>
+      </c>
+      <c r="X11" t="n">
+        <v>283.3109225452652</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>266.0766365969678</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>300.5452084935625</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>262.9659924470926</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>308.7710052490234</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>122</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>31.21898795984968</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>38.15980777324834</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>34.49176155124631</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>34.42623029342849</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>1.777300376160677</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>32.13088525699663</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>36.91245386750294</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>1.133343848778651</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.8114754098360656</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>257.8688405483584</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>315.2000122070312</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>284.9019504132945</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>270.2214493062074</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>299.5824515203817</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>265.4011122227922</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>304.8968689455743</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Advanced Micro Devices, Inc.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>490.33</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="J12" t="n">
+        <v>163.98996</v>
+      </c>
+      <c r="K12" t="n">
+        <v>63</v>
+      </c>
+      <c r="L12" t="n">
+        <v>62</v>
+      </c>
+      <c r="M12" t="n">
+        <v>72.9773582602447</v>
+      </c>
+      <c r="N12" t="n">
+        <v>177.8754162397541</v>
+      </c>
+      <c r="O12" t="n">
+        <v>117.0632143411623</v>
+      </c>
+      <c r="P12" t="n">
+        <v>118.5924486844045</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>34.08285792004858</v>
+      </c>
+      <c r="R12" t="n">
+        <v>75.99849139519458</v>
+      </c>
+      <c r="S12" t="n">
+        <v>164.9360701764216</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1.3768430384834</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.8870967741935484</v>
+      </c>
+      <c r="V12" t="n">
+        <v>218.2023011981317</v>
+      </c>
+      <c r="W12" t="n">
+        <v>531.8474945568648</v>
+      </c>
+      <c r="X12" t="n">
+        <v>350.0190108800753</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>248.11126569913</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>451.9267560610205</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>227.2354892716318</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>493.1588498275007</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>122</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>72.05660262197819</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>177.8754162397541</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>107.2228551603934</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>105.0953815714424</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>29.0980349864215</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>75.51811131891215</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>149.0626240714652</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>1.950891352838665</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0.9426229508196722</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>215.4492418397148</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>531.8474945568648</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>320.5963369295761</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>233.5932123201758</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>407.5994615389765</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>225.7991528435473</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>445.6972459736809</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>245.22</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="J13" t="n">
+        <v>31.64129</v>
+      </c>
+      <c r="K13" t="n">
+        <v>67</v>
+      </c>
+      <c r="L13" t="n">
+        <v>62</v>
+      </c>
+      <c r="M13" t="n">
+        <v>27.80195206944081</v>
+      </c>
+      <c r="N13" t="n">
+        <v>36.81868761985704</v>
+      </c>
+      <c r="O13" t="n">
+        <v>31.70656586892432</v>
+      </c>
+      <c r="P13" t="n">
+        <v>31.71949797269831</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>2.364655164592175</v>
+      </c>
+      <c r="R13" t="n">
+        <v>29.05425429510439</v>
+      </c>
+      <c r="S13" t="n">
+        <v>34.93654088827689</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-0.02760481523976249</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.4516129032258064</v>
+      </c>
+      <c r="V13" t="n">
+        <v>215.4651285381663</v>
+      </c>
+      <c r="W13" t="n">
+        <v>285.3448290538921</v>
+      </c>
+      <c r="X13" t="n">
+        <v>245.7258854841635</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>227.3998079585741</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>264.0519630097529</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>225.170470787059</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>270.758191884146</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>122</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>27.72524313614126</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>36.81868761985704</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>31.6787340441008</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>31.95592771818937</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>2.268451172495901</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>28.94741893645942</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>34.72357096864921</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>-0.01650643600126667</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>0.4426229508196721</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>214.8706343050948</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>285.3448290538921</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>245.5101888417812</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>227.929692254938</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>263.0906854286245</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>224.3424967575606</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>269.1076750070314</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>396.6</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="J14" t="n">
+        <v>65.77114</v>
+      </c>
+      <c r="K14" t="n">
+        <v>33</v>
+      </c>
+      <c r="L14" t="n">
+        <v>62</v>
+      </c>
+      <c r="M14" t="n">
+        <v>57.19493248774063</v>
+      </c>
+      <c r="N14" t="n">
+        <v>93.87329577470153</v>
+      </c>
+      <c r="O14" t="n">
+        <v>75.04499179120712</v>
+      </c>
+      <c r="P14" t="n">
+        <v>78.71540210865163</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>9.781241462981987</v>
+      </c>
+      <c r="R14" t="n">
+        <v>61.29473531920079</v>
+      </c>
+      <c r="S14" t="n">
+        <v>83.49376061274063</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-0.9481262502622875</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.2903225806451613</v>
+      </c>
+      <c r="V14" t="n">
+        <v>344.885442901076</v>
+      </c>
+      <c r="W14" t="n">
+        <v>566.0559735214503</v>
+      </c>
+      <c r="X14" t="n">
+        <v>452.521300500979</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>393.5404144791976</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>511.5021865227603</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>369.6072539747808</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>503.467376494826</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>117</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>57.19493248774063</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>93.87329577470153</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>72.76569347655681</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>71.85744439530923</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>7.673032529667959</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>62.51890781097711</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>82.39649127566095</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>-0.9115761531717999</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0.1709401709401709</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>344.885442901076</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>566.0559735214503</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>438.7771316636375</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>392.5087455097398</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>485.0455178175354</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>376.989014100192</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>496.8508423922356</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>361.17</v>
+      </c>
+      <c r="I15" t="n">
+        <v>13.11</v>
+      </c>
+      <c r="J15" t="n">
+        <v>27.5492</v>
+      </c>
+      <c r="K15" t="n">
+        <v>37</v>
+      </c>
+      <c r="L15" t="n">
+        <v>62</v>
+      </c>
+      <c r="M15" t="n">
+        <v>25.26734640596091</v>
+      </c>
+      <c r="N15" t="n">
+        <v>32.24051702254134</v>
+      </c>
+      <c r="O15" t="n">
+        <v>29.0332733400003</v>
+      </c>
+      <c r="P15" t="n">
+        <v>29.21870597964289</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.623880269917904</v>
+      </c>
+      <c r="R15" t="n">
+        <v>27.14135001944186</v>
+      </c>
+      <c r="S15" t="n">
+        <v>31.22081491927324</v>
+      </c>
+      <c r="T15" t="n">
+        <v>-0.9139056416242591</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.1774193548387097</v>
+      </c>
+      <c r="V15" t="n">
+        <v>331.2549113821476</v>
+      </c>
+      <c r="W15" t="n">
+        <v>422.673178165517</v>
+      </c>
+      <c r="X15" t="n">
+        <v>380.6262134874038</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>359.3371431487801</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>401.9152838260276</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>355.8230987548828</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>409.3048835916722</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>122</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>25.26734640596091</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>34.04738340537852</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>29.83504690282757</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>29.46390610450698</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>1.933208796634226</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>27.59935151416874</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>32.65449124757065</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>-1.182410770532027</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0.09016393442622951</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>331.2549113821476</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>446.3611964445124</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>391.1374648960694</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>365.7930975721947</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>416.4818322199441</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>361.8274983507521</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>428.1003802556511</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>585.39</v>
+      </c>
+      <c r="I16" t="n">
+        <v>27.51</v>
+      </c>
+      <c r="J16" t="n">
+        <v>21.279171</v>
+      </c>
+      <c r="K16" t="n">
+        <v>55</v>
+      </c>
+      <c r="L16" t="n">
+        <v>62</v>
+      </c>
+      <c r="M16" t="n">
+        <v>21.28690962357955</v>
+      </c>
+      <c r="N16" t="n">
+        <v>29.31247287326389</v>
+      </c>
+      <c r="O16" t="n">
+        <v>24.6634695409604</v>
+      </c>
+      <c r="P16" t="n">
+        <v>24.37526659033764</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>2.603320992855815</v>
+      </c>
+      <c r="R16" t="n">
+        <v>21.93440007990057</v>
+      </c>
+      <c r="S16" t="n">
+        <v>28.57799154893039</v>
+      </c>
+      <c r="T16" t="n">
+        <v>-1.299992797756324</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>585.6028837446734</v>
+      </c>
+      <c r="W16" t="n">
+        <v>806.3861287434895</v>
+      </c>
+      <c r="X16" t="n">
+        <v>678.4920470718207</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>606.8746865583573</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>750.1094075852842</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>603.4153461980646</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>786.1805475110751</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>122</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>21.28690962357955</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>31.43082152229007</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>26.56178868730787</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>27.52679771768262</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>2.759774229104261</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>22.19181840376421</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>29.31080928832899</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>-1.914148495046441</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>585.6028837446734</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>864.6619000781998</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>730.7148067878396</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>654.7934177451815</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>806.6361958304979</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>610.4969242875534</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>806.3403635219306</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>411.74</v>
+      </c>
+      <c r="I17" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="J17" t="n">
+        <v>24.508333</v>
+      </c>
+      <c r="K17" t="n">
+        <v>67</v>
+      </c>
+      <c r="L17" t="n">
+        <v>62</v>
+      </c>
+      <c r="M17" t="n">
+        <v>22.31206935670243</v>
+      </c>
+      <c r="N17" t="n">
+        <v>27.41190410795666</v>
+      </c>
+      <c r="O17" t="n">
+        <v>24.76636544625846</v>
+      </c>
+      <c r="P17" t="n">
+        <v>24.72342929518021</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1.186495357009306</v>
+      </c>
+      <c r="R17" t="n">
+        <v>23.21232073451669</v>
+      </c>
+      <c r="S17" t="n">
+        <v>26.51801151659729</v>
+      </c>
+      <c r="T17" t="n">
+        <v>-0.2174744677542248</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0.3870967741935484</v>
+      </c>
+      <c r="V17" t="n">
+        <v>374.8427651926008</v>
+      </c>
+      <c r="W17" t="n">
+        <v>460.5199890136719</v>
+      </c>
+      <c r="X17" t="n">
+        <v>416.0749394971421</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>396.1418174993858</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>436.0080614948985</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>389.9669883398803</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>445.5025934788345</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>122</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>22.31206935670243</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>34.70981429684721</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>27.23040246766649</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>25.30487804878049</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>3.996590461513518</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>23.45741009548204</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>34.08285908814344</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>-0.6810979243131255</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>0.2131147540983606</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>374.8427651926008</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>583.1248801870332</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>457.4707614567971</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>390.32804170337</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>524.6134812102242</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>394.0844896040983</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>572.5920326808099</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>82.64</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>26.658066</v>
+      </c>
+      <c r="K18" t="n">
+        <v>67</v>
+      </c>
+      <c r="L18" t="n">
+        <v>26</v>
+      </c>
+      <c r="M18" t="n">
+        <v>35.93675816954359</v>
+      </c>
+      <c r="N18" t="n">
+        <v>42.60474344487245</v>
+      </c>
+      <c r="O18" t="n">
+        <v>38.40270594790844</v>
+      </c>
+      <c r="P18" t="n">
+        <v>37.65019654285294</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1.990322096160243</v>
+      </c>
+      <c r="R18" t="n">
+        <v>36.38339890792905</v>
+      </c>
+      <c r="S18" t="n">
+        <v>41.39130483031742</v>
+      </c>
+      <c r="T18" t="n">
+        <v>-5.900874019620422</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>111.4039503255851</v>
+      </c>
+      <c r="W18" t="n">
+        <v>132.0747046791046</v>
+      </c>
+      <c r="X18" t="n">
+        <v>119.0483884385162</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>112.8783899404194</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>125.2183869366129</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>112.7885366145801</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>128.313044973984</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>86</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>3.489557264641911</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>42.60474344487245</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>25.3821414425773</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>32.59090830686063</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>15.350467123509</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>3.777151179492922</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>39.12055275656958</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0.08311959155097284</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>0.3255813953488372</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>10.81762752038992</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>132.0747046791046</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>78.68463847198962</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>31.09819038911171</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>126.2710865548675</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>11.70916865642806</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>121.2737135453657</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:47:43</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SEC point-in-time</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>208.64</v>
+      </c>
+      <c r="I19" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="J19" t="n">
+        <v>31.950994</v>
+      </c>
+      <c r="K19" t="n">
+        <v>65</v>
+      </c>
+      <c r="L19" t="n">
+        <v>62</v>
+      </c>
+      <c r="M19" t="n">
+        <v>31.4088830173837</v>
+      </c>
+      <c r="N19" t="n">
+        <v>48.11020520268654</v>
+      </c>
+      <c r="O19" t="n">
+        <v>38.36880050331563</v>
+      </c>
+      <c r="P19" t="n">
+        <v>37.38367353166852</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>4.287242152477702</v>
+      </c>
+      <c r="R19" t="n">
+        <v>32.91071986713963</v>
+      </c>
+      <c r="S19" t="n">
+        <v>44.72591882822464</v>
+      </c>
+      <c r="T19" t="n">
+        <v>-1.496954516461501</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.01612903225806452</v>
+      </c>
+      <c r="V19" t="n">
+        <v>205.1000061035156</v>
+      </c>
+      <c r="W19" t="n">
+        <v>314.1596399735431</v>
+      </c>
+      <c r="X19" t="n">
+        <v>250.5482672866511</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>222.5525760309716</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>278.5439585423305</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>214.9070007324218</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>292.0602499483069</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>72</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>31.4088830173837</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>48.11020520268654</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>38.23194894045754</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>37.36530537507971</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>4.00582481027654</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>33.02649341717613</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>44.17734698860012</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>-1.567955474324383</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0.01388888888888889</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>205.1000061035156</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>314.1596399735431</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>249.6546265811877</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>223.4965905700819</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>275.8126625922935</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>215.6630020141602</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>288.4780758355588</v>
       </c>
     </row>
   </sheetData>
@@ -2247,12 +3606,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2281,19 +3640,19 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>365.76</v>
+        <v>361.17</v>
       </c>
       <c r="I2" t="n">
-        <v>13.09</v>
+        <v>13.11</v>
       </c>
       <c r="J2" t="n">
-        <v>27.94194</v>
+        <v>27.5492</v>
       </c>
       <c r="K2" t="n">
         <v>37</v>
       </c>
       <c r="L2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M2" t="n">
         <v>25.26734640596091</v>
@@ -2302,49 +3661,49 @@
         <v>32.24051702254134</v>
       </c>
       <c r="O2" t="n">
-        <v>29.03515793312945</v>
+        <v>29.0332733400003</v>
       </c>
       <c r="P2" t="n">
-        <v>29.20629058470889</v>
+        <v>29.21870597964289</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.604375173463596</v>
+        <v>1.623880269917904</v>
       </c>
       <c r="R2" t="n">
-        <v>27.15226581494923</v>
+        <v>27.14135001944186</v>
       </c>
       <c r="S2" t="n">
-        <v>31.19926064462159</v>
+        <v>31.22081491927324</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.6813979368487536</v>
+        <v>-0.9139056416242591</v>
       </c>
       <c r="U2" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="V2" t="n">
-        <v>330.7495644540284</v>
+        <v>331.2549113821476</v>
       </c>
       <c r="W2" t="n">
-        <v>422.0283678250661</v>
+        <v>422.673178165517</v>
       </c>
       <c r="X2" t="n">
-        <v>380.0702173446646</v>
+        <v>380.6262134874038</v>
       </c>
       <c r="Y2" t="n">
-        <v>359.0689463240261</v>
+        <v>359.3371431487801</v>
       </c>
       <c r="Z2" t="n">
-        <v>401.071488365303</v>
+        <v>401.9152838260276</v>
       </c>
       <c r="AA2" t="n">
-        <v>355.4231595176854</v>
+        <v>355.8230987548828</v>
       </c>
       <c r="AB2" t="n">
-        <v>408.3983218380966</v>
+        <v>409.3048835916722</v>
       </c>
       <c r="AC2" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD2" t="n">
         <v>25.26734640596091</v>
@@ -2353,57 +3712,57 @@
         <v>34.04738340537852</v>
       </c>
       <c r="AF2" t="n">
-        <v>29.89051020637544</v>
+        <v>29.83504690282757</v>
       </c>
       <c r="AG2" t="n">
-        <v>29.51552249913338</v>
+        <v>29.46390610450698</v>
       </c>
       <c r="AH2" t="n">
-        <v>1.920880039883152</v>
+        <v>1.933208796634226</v>
       </c>
       <c r="AI2" t="n">
-        <v>27.64653123825595</v>
+        <v>27.59935151416874</v>
       </c>
       <c r="AJ2" t="n">
-        <v>32.6446195792587</v>
+        <v>32.65449124757065</v>
       </c>
       <c r="AK2" t="n">
-        <v>-1.014415354377868</v>
+        <v>-1.182410770532027</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.1370967741935484</v>
+        <v>0.09016393442622951</v>
       </c>
       <c r="AM2" t="n">
-        <v>330.7495644540284</v>
+        <v>331.2549113821476</v>
       </c>
       <c r="AN2" t="n">
-        <v>445.6802487764048</v>
+        <v>446.3611964445124</v>
       </c>
       <c r="AO2" t="n">
-        <v>391.2667786014545</v>
+        <v>391.1374648960694</v>
       </c>
       <c r="AP2" t="n">
-        <v>366.1224588793841</v>
+        <v>365.7930975721947</v>
       </c>
       <c r="AQ2" t="n">
-        <v>416.4110983235249</v>
+        <v>416.4818322199441</v>
       </c>
       <c r="AR2" t="n">
-        <v>361.8930939087704</v>
+        <v>361.8274983507521</v>
       </c>
       <c r="AS2" t="n">
-        <v>427.3180702924964</v>
+        <v>428.1003802556511</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2432,19 +3791,19 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>416.67</v>
+        <v>411.74</v>
       </c>
       <c r="I3" t="n">
-        <v>16.78</v>
+        <v>16.8</v>
       </c>
       <c r="J3" t="n">
-        <v>24.831347</v>
+        <v>24.508333</v>
       </c>
       <c r="K3" t="n">
         <v>67</v>
       </c>
       <c r="L3" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M3" t="n">
         <v>22.31206935670243</v>
@@ -2453,108 +3812,108 @@
         <v>27.41190410795666</v>
       </c>
       <c r="O3" t="n">
-        <v>24.79343354361776</v>
+        <v>24.76636544625846</v>
       </c>
       <c r="P3" t="n">
-        <v>24.76369040352958</v>
+        <v>24.72342929518021</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.183451999371762</v>
+        <v>1.186495357009306</v>
       </c>
       <c r="R3" t="n">
-        <v>23.22013812038286</v>
+        <v>23.21232073451669</v>
       </c>
       <c r="S3" t="n">
-        <v>26.50944369222463</v>
+        <v>26.51801151659729</v>
       </c>
       <c r="T3" t="n">
-        <v>0.03203632796460248</v>
+        <v>-0.2174744677542248</v>
       </c>
       <c r="U3" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="V3" t="n">
-        <v>374.3965238054668</v>
+        <v>374.8427651926008</v>
       </c>
       <c r="W3" t="n">
-        <v>459.9717509315128</v>
+        <v>460.5199890136719</v>
       </c>
       <c r="X3" t="n">
-        <v>416.0338148619061</v>
+        <v>416.0749394971421</v>
       </c>
       <c r="Y3" t="n">
-        <v>396.1754903124479</v>
+        <v>396.1418174993858</v>
       </c>
       <c r="Z3" t="n">
-        <v>435.8921394113643</v>
+        <v>436.0080614948985</v>
       </c>
       <c r="AA3" t="n">
-        <v>389.6339176600243</v>
+        <v>389.9669883398803</v>
       </c>
       <c r="AB3" t="n">
-        <v>444.8284651555294</v>
+        <v>445.5025934788345</v>
       </c>
       <c r="AC3" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD3" t="n">
         <v>22.31206935670243</v>
       </c>
       <c r="AE3" t="n">
-        <v>34.99430931818434</v>
+        <v>34.70981429684721</v>
       </c>
       <c r="AF3" t="n">
-        <v>27.43189715615672</v>
+        <v>27.23040246766649</v>
       </c>
       <c r="AG3" t="n">
-        <v>25.35834965517999</v>
+        <v>25.30487804878049</v>
       </c>
       <c r="AH3" t="n">
-        <v>4.118216138579381</v>
+        <v>3.996590461513518</v>
       </c>
       <c r="AI3" t="n">
-        <v>23.55171914544979</v>
+        <v>23.45741009548204</v>
       </c>
       <c r="AJ3" t="n">
-        <v>34.32453746985575</v>
+        <v>34.08285908814344</v>
       </c>
       <c r="AK3" t="n">
-        <v>-0.6314749077385238</v>
+        <v>-0.6810979243131255</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.3064516129032258</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="AM3" t="n">
-        <v>374.3965238054668</v>
+        <v>374.8427651926008</v>
       </c>
       <c r="AN3" t="n">
-        <v>587.2045103591333</v>
+        <v>583.1248801870332</v>
       </c>
       <c r="AO3" t="n">
-        <v>460.3072342803097</v>
+        <v>457.4707614567971</v>
       </c>
       <c r="AP3" t="n">
-        <v>391.2035674749477</v>
+        <v>390.32804170337</v>
       </c>
       <c r="AQ3" t="n">
-        <v>529.4109010856718</v>
+        <v>524.6134812102242</v>
       </c>
       <c r="AR3" t="n">
-        <v>395.1978472606475</v>
+        <v>394.0844896040983</v>
       </c>
       <c r="AS3" t="n">
-        <v>575.9657387441795</v>
+        <v>572.5920326808099</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2583,129 +3942,129 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>593</v>
+        <v>585.39</v>
       </c>
       <c r="I4" t="n">
-        <v>27.52</v>
+        <v>27.51</v>
       </c>
       <c r="J4" t="n">
-        <v>21.547964</v>
+        <v>21.279171</v>
       </c>
       <c r="K4" t="n">
         <v>55</v>
       </c>
       <c r="L4" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M4" t="n">
-        <v>21.56363636363636</v>
+        <v>21.28690962357955</v>
       </c>
       <c r="N4" t="n">
         <v>29.31247287326389</v>
       </c>
       <c r="O4" t="n">
-        <v>24.81354057111685</v>
+        <v>24.6634695409604</v>
       </c>
       <c r="P4" t="n">
-        <v>24.45551391965331</v>
+        <v>24.37526659033764</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.599953635337401</v>
+        <v>2.603320992855815</v>
       </c>
       <c r="R4" t="n">
-        <v>21.99927334872159</v>
+        <v>21.93440007990057</v>
       </c>
       <c r="S4" t="n">
-        <v>28.57616075407753</v>
+        <v>28.57799154893039</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.256013386828365</v>
+        <v>-1.299992797756324</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>593.4312727272727</v>
+        <v>585.6028837446734</v>
       </c>
       <c r="W4" t="n">
-        <v>806.6792534722222</v>
+        <v>806.3861287434895</v>
       </c>
       <c r="X4" t="n">
-        <v>682.8686365171357</v>
+        <v>678.4920470718207</v>
       </c>
       <c r="Y4" t="n">
-        <v>611.3179124726504</v>
+        <v>606.8746865583573</v>
       </c>
       <c r="Z4" t="n">
-        <v>754.4193605616209</v>
+        <v>750.1094075852842</v>
       </c>
       <c r="AA4" t="n">
-        <v>605.4200025568182</v>
+        <v>603.4153461980646</v>
       </c>
       <c r="AB4" t="n">
-        <v>786.4159439522136</v>
+        <v>786.1805475110751</v>
       </c>
       <c r="AC4" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD4" t="n">
-        <v>21.56363636363636</v>
+        <v>21.28690962357955</v>
       </c>
       <c r="AE4" t="n">
         <v>31.43082152229007</v>
       </c>
       <c r="AF4" t="n">
-        <v>26.66668497656942</v>
+        <v>26.56178868730787</v>
       </c>
       <c r="AG4" t="n">
-        <v>27.62856513908844</v>
+        <v>27.52679771768262</v>
       </c>
       <c r="AH4" t="n">
-        <v>2.723870427428682</v>
+        <v>2.759774229104261</v>
       </c>
       <c r="AI4" t="n">
-        <v>22.2054541015625</v>
+        <v>22.19181840376421</v>
       </c>
       <c r="AJ4" t="n">
-        <v>29.35631868302171</v>
+        <v>29.31080928832899</v>
       </c>
       <c r="AK4" t="n">
-        <v>-1.879208689600359</v>
+        <v>-1.914148495046441</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>593.4312727272727</v>
+        <v>585.6028837446734</v>
       </c>
       <c r="AN4" t="n">
-        <v>864.9762082934226</v>
+        <v>864.6619000781998</v>
       </c>
       <c r="AO4" t="n">
-        <v>733.8671705551906</v>
+        <v>730.7148067878396</v>
       </c>
       <c r="AP4" t="n">
-        <v>658.9062563923532</v>
+        <v>654.7934177451815</v>
       </c>
       <c r="AQ4" t="n">
-        <v>808.8280847180279</v>
+        <v>806.6361958304979</v>
       </c>
       <c r="AR4" t="n">
-        <v>611.094096875</v>
+        <v>610.4969242875534</v>
       </c>
       <c r="AS4" t="n">
-        <v>807.8858901567575</v>
+        <v>806.3403635219306</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2734,19 +4093,19 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>246.03</v>
+        <v>245.22</v>
       </c>
       <c r="I5" t="n">
-        <v>7.77</v>
+        <v>7.75</v>
       </c>
       <c r="J5" t="n">
-        <v>31.664093</v>
+        <v>31.64129</v>
       </c>
       <c r="K5" t="n">
         <v>67</v>
       </c>
       <c r="L5" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M5" t="n">
         <v>27.80195206944081</v>
@@ -2755,49 +4114,49 @@
         <v>36.81868761985704</v>
       </c>
       <c r="O5" t="n">
-        <v>31.68480333699108</v>
+        <v>31.70656586892432</v>
       </c>
       <c r="P5" t="n">
-        <v>31.70574133476002</v>
+        <v>31.71949797269831</v>
       </c>
       <c r="Q5" t="n">
-        <v>2.350157910663178</v>
+        <v>2.364655164592175</v>
       </c>
       <c r="R5" t="n">
-        <v>29.0610881895866</v>
+        <v>29.05425429510439</v>
       </c>
       <c r="S5" t="n">
-        <v>34.92747542249608</v>
+        <v>34.93654088827689</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.00881231720520243</v>
+        <v>-0.02760481523976249</v>
       </c>
       <c r="U5" t="n">
-        <v>0.4603174603174603</v>
+        <v>0.4516129032258064</v>
       </c>
       <c r="V5" t="n">
-        <v>216.0211675795551</v>
+        <v>215.4651285381663</v>
       </c>
       <c r="W5" t="n">
-        <v>286.0812028062892</v>
+        <v>285.3448290538921</v>
       </c>
       <c r="X5" t="n">
-        <v>246.1909219284207</v>
+        <v>245.7258854841635</v>
       </c>
       <c r="Y5" t="n">
-        <v>227.9301949625678</v>
+        <v>227.3998079585741</v>
       </c>
       <c r="Z5" t="n">
-        <v>264.4516488942736</v>
+        <v>264.0519630097529</v>
       </c>
       <c r="AA5" t="n">
-        <v>225.8046552330879</v>
+        <v>225.170470787059</v>
       </c>
       <c r="AB5" t="n">
-        <v>271.3864840327946</v>
+        <v>270.758191884146</v>
       </c>
       <c r="AC5" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD5" t="n">
         <v>27.72524313614126</v>
@@ -2806,57 +4165,57 @@
         <v>36.81868761985704</v>
       </c>
       <c r="AF5" t="n">
-        <v>31.71329843171316</v>
+        <v>31.6787340441008</v>
       </c>
       <c r="AG5" t="n">
-        <v>32.0098866177144</v>
+        <v>31.95592771818937</v>
       </c>
       <c r="AH5" t="n">
-        <v>2.242452514636653</v>
+        <v>2.268451172495901</v>
       </c>
       <c r="AI5" t="n">
-        <v>28.95104529302323</v>
+        <v>28.94741893645942</v>
       </c>
       <c r="AJ5" t="n">
-        <v>34.70906596802268</v>
+        <v>34.72357096864921</v>
       </c>
       <c r="AK5" t="n">
-        <v>-0.02194268614028044</v>
+        <v>-0.01650643600126667</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.4274193548387097</v>
+        <v>0.4426229508196721</v>
       </c>
       <c r="AM5" t="n">
-        <v>215.4251391678176</v>
+        <v>214.8706343050948</v>
       </c>
       <c r="AN5" t="n">
-        <v>286.0812028062892</v>
+        <v>285.3448290538921</v>
       </c>
       <c r="AO5" t="n">
-        <v>246.4123288144112</v>
+        <v>245.5101888417812</v>
       </c>
       <c r="AP5" t="n">
-        <v>228.9884727756844</v>
+        <v>227.929692254938</v>
       </c>
       <c r="AQ5" t="n">
-        <v>263.836184853138</v>
+        <v>263.0906854286245</v>
       </c>
       <c r="AR5" t="n">
-        <v>224.9496219267905</v>
+        <v>224.3424967575606</v>
       </c>
       <c r="AS5" t="n">
-        <v>269.6894425715362</v>
+        <v>269.1076750070314</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2885,19 +4244,19 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>307.34</v>
+        <v>301.54</v>
       </c>
       <c r="I6" t="n">
-        <v>8.27</v>
+        <v>8.26</v>
       </c>
       <c r="J6" t="n">
-        <v>37.16324</v>
+        <v>36.506054</v>
       </c>
       <c r="K6" t="n">
         <v>67</v>
       </c>
       <c r="L6" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M6" t="n">
         <v>31.21898795984968</v>
@@ -2906,49 +4265,49 @@
         <v>38.15980777324834</v>
       </c>
       <c r="O6" t="n">
-        <v>34.22148379509058</v>
+        <v>34.29914316528635</v>
       </c>
       <c r="P6" t="n">
-        <v>33.91525601070672</v>
+        <v>34.20253319076345</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.063192221013672</v>
+        <v>2.086475296404038</v>
       </c>
       <c r="R6" t="n">
-        <v>31.83797522436215</v>
+        <v>31.83607656744462</v>
       </c>
       <c r="S6" t="n">
-        <v>37.37554517842955</v>
+        <v>37.38147763305368</v>
       </c>
       <c r="T6" t="n">
-        <v>1.425827499225494</v>
+        <v>1.057722005392147</v>
       </c>
       <c r="U6" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.7903225806451613</v>
       </c>
       <c r="V6" t="n">
-        <v>258.1810304279569</v>
+        <v>257.8688405483584</v>
       </c>
       <c r="W6" t="n">
-        <v>315.5816102847638</v>
+        <v>315.2000122070312</v>
       </c>
       <c r="X6" t="n">
-        <v>283.0116709853991</v>
+        <v>283.3109225452652</v>
       </c>
       <c r="Y6" t="n">
-        <v>265.9490713176161</v>
+        <v>266.0766365969678</v>
       </c>
       <c r="Z6" t="n">
-        <v>300.0742706531822</v>
+        <v>300.5452084935625</v>
       </c>
       <c r="AA6" t="n">
-        <v>263.3000551054749</v>
+        <v>262.9659924470926</v>
       </c>
       <c r="AB6" t="n">
-        <v>309.0957586256124</v>
+        <v>308.7710052490234</v>
       </c>
       <c r="AC6" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD6" t="n">
         <v>31.21898795984968</v>
@@ -2957,57 +4316,57 @@
         <v>38.15980777324834</v>
       </c>
       <c r="AF6" t="n">
-        <v>34.54245963852536</v>
+        <v>34.49176155124631</v>
       </c>
       <c r="AG6" t="n">
-        <v>34.49936878832081</v>
+        <v>34.42623029342849</v>
       </c>
       <c r="AH6" t="n">
-        <v>1.805208059622547</v>
+        <v>1.777300376160677</v>
       </c>
       <c r="AI6" t="n">
-        <v>32.14202455931072</v>
+        <v>32.13088525699663</v>
       </c>
       <c r="AJ6" t="n">
-        <v>37.19241090054221</v>
+        <v>36.91245386750294</v>
       </c>
       <c r="AK6" t="n">
-        <v>1.451788533462799</v>
+        <v>1.133343848778651</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.8951612903225806</v>
+        <v>0.8114754098360656</v>
       </c>
       <c r="AM6" t="n">
-        <v>258.1810304279569</v>
+        <v>257.8688405483584</v>
       </c>
       <c r="AN6" t="n">
-        <v>315.5816102847638</v>
+        <v>315.2000122070312</v>
       </c>
       <c r="AO6" t="n">
-        <v>285.6661412106047</v>
+        <v>284.9019504132945</v>
       </c>
       <c r="AP6" t="n">
-        <v>270.7370705575262</v>
+        <v>270.2214493062074</v>
       </c>
       <c r="AQ6" t="n">
-        <v>300.5952118636832</v>
+        <v>299.5824515203817</v>
       </c>
       <c r="AR6" t="n">
-        <v>265.8145431054996</v>
+        <v>265.4011122227922</v>
       </c>
       <c r="AS6" t="n">
-        <v>307.5812381474841</v>
+        <v>304.8968689455743</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3036,19 +4395,19 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>205.1</v>
+        <v>208.64</v>
       </c>
       <c r="I7" t="n">
-        <v>6.52</v>
+        <v>6.53</v>
       </c>
       <c r="J7" t="n">
-        <v>31.457056</v>
+        <v>31.950994</v>
       </c>
       <c r="K7" t="n">
         <v>65</v>
       </c>
       <c r="L7" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M7" t="n">
         <v>31.4088830173837</v>
@@ -3057,49 +4416,49 @@
         <v>48.11020520268654</v>
       </c>
       <c r="O7" t="n">
-        <v>38.44283030141145</v>
+        <v>38.36880050331563</v>
       </c>
       <c r="P7" t="n">
-        <v>37.39183698381696</v>
+        <v>37.38367353166852</v>
       </c>
       <c r="Q7" t="n">
-        <v>4.176171651630198</v>
+        <v>4.287242152477702</v>
       </c>
       <c r="R7" t="n">
-        <v>33.07748885103608</v>
+        <v>32.91071986713963</v>
       </c>
       <c r="S7" t="n">
-        <v>44.66816368881537</v>
+        <v>44.72591882822464</v>
       </c>
       <c r="T7" t="n">
-        <v>-1.672769915643793</v>
+        <v>-1.496954516461501</v>
       </c>
       <c r="U7" t="n">
-        <v>0.01587301587301587</v>
+        <v>0.01612903225806452</v>
       </c>
       <c r="V7" t="n">
-        <v>204.7859172733417</v>
+        <v>205.1000061035156</v>
       </c>
       <c r="W7" t="n">
-        <v>313.6785379215162</v>
+        <v>314.1596399735431</v>
       </c>
       <c r="X7" t="n">
-        <v>250.6472535652026</v>
+        <v>250.5482672866511</v>
       </c>
       <c r="Y7" t="n">
-        <v>223.4186143965737</v>
+        <v>222.5525760309716</v>
       </c>
       <c r="Z7" t="n">
-        <v>277.8758927338315</v>
+        <v>278.5439585423305</v>
       </c>
       <c r="AA7" t="n">
-        <v>215.6652273087552</v>
+        <v>214.9070007324218</v>
       </c>
       <c r="AB7" t="n">
-        <v>291.2364272510762</v>
+        <v>292.0602499483069</v>
       </c>
       <c r="AC7" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AD7" t="n">
         <v>31.4088830173837</v>
@@ -3108,57 +4467,57 @@
         <v>48.11020520268654</v>
       </c>
       <c r="AF7" t="n">
-        <v>38.32041307606467</v>
+        <v>38.23194894045754</v>
       </c>
       <c r="AG7" t="n">
-        <v>37.37551007952008</v>
+        <v>37.36530537507971</v>
       </c>
       <c r="AH7" t="n">
-        <v>3.962872125009824</v>
+        <v>4.00582481027654</v>
       </c>
       <c r="AI7" t="n">
-        <v>33.48545232191567</v>
+        <v>33.02649341717613</v>
       </c>
       <c r="AJ7" t="n">
-        <v>44.20612257354113</v>
+        <v>44.17734698860012</v>
       </c>
       <c r="AK7" t="n">
-        <v>-1.731914848513478</v>
+        <v>-1.567955474324383</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.01408450704225352</v>
+        <v>0.01388888888888889</v>
       </c>
       <c r="AM7" t="n">
-        <v>204.7859172733417</v>
+        <v>205.1000061035156</v>
       </c>
       <c r="AN7" t="n">
-        <v>313.6785379215162</v>
+        <v>314.1596399735431</v>
       </c>
       <c r="AO7" t="n">
-        <v>249.8490932559417</v>
+        <v>249.6546265811877</v>
       </c>
       <c r="AP7" t="n">
-        <v>224.0111670008776</v>
+        <v>223.4965905700819</v>
       </c>
       <c r="AQ7" t="n">
-        <v>275.6870195110057</v>
+        <v>275.8126625922935</v>
       </c>
       <c r="AR7" t="n">
-        <v>218.3251491388902</v>
+        <v>215.6630020141602</v>
       </c>
       <c r="AS7" t="n">
-        <v>288.2239191794881</v>
+        <v>288.4780758355588</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3187,19 +4546,19 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>466.38</v>
+        <v>490.33</v>
       </c>
       <c r="I8" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="J8" t="n">
-        <v>156.50336</v>
+        <v>163.98996</v>
       </c>
       <c r="K8" t="n">
         <v>63</v>
       </c>
       <c r="L8" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M8" t="n">
         <v>72.9773582602447</v>
@@ -3208,49 +4567,49 @@
         <v>177.8754162397541</v>
       </c>
       <c r="O8" t="n">
-        <v>115.0845863437765</v>
+        <v>117.0632143411623</v>
       </c>
       <c r="P8" t="n">
-        <v>114.513204322671</v>
+        <v>118.5924486844045</v>
       </c>
       <c r="Q8" t="n">
-        <v>34.07307640454155</v>
+        <v>34.08285792004858</v>
       </c>
       <c r="R8" t="n">
-        <v>76.02339719376475</v>
+        <v>75.99849139519458</v>
       </c>
       <c r="S8" t="n">
-        <v>164.6622994845031</v>
+        <v>164.9360701764216</v>
       </c>
       <c r="T8" t="n">
-        <v>1.215586557681737</v>
+        <v>1.3768430384834</v>
       </c>
       <c r="U8" t="n">
-        <v>0.873015873015873</v>
+        <v>0.8870967741935484</v>
       </c>
       <c r="V8" t="n">
-        <v>217.4725276155292</v>
+        <v>218.2023011981317</v>
       </c>
       <c r="W8" t="n">
-        <v>530.0687403944672</v>
+        <v>531.8474945568648</v>
       </c>
       <c r="X8" t="n">
-        <v>342.952067304454</v>
+        <v>350.0190108800753</v>
       </c>
       <c r="Y8" t="n">
-        <v>241.4142996189202</v>
+        <v>248.11126569913</v>
       </c>
       <c r="Z8" t="n">
-        <v>444.4898349899879</v>
+        <v>451.9267560610205</v>
       </c>
       <c r="AA8" t="n">
-        <v>226.549723637419</v>
+        <v>227.2354892716318</v>
       </c>
       <c r="AB8" t="n">
-        <v>490.6936524638191</v>
+        <v>493.1588498275007</v>
       </c>
       <c r="AC8" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AD8" t="n">
         <v>72.05660262197819</v>
@@ -3259,57 +4618,57 @@
         <v>177.8754162397541</v>
       </c>
       <c r="AF8" t="n">
-        <v>106.8354184211481</v>
+        <v>107.2228551603934</v>
       </c>
       <c r="AG8" t="n">
-        <v>105.3177330881504</v>
+        <v>105.0953815714424</v>
       </c>
       <c r="AH8" t="n">
-        <v>28.45264556448733</v>
+        <v>29.0980349864215</v>
       </c>
       <c r="AI8" t="n">
-        <v>75.52037537772701</v>
+        <v>75.51811131891215</v>
       </c>
       <c r="AJ8" t="n">
-        <v>147.4318057200948</v>
+        <v>149.0626240714652</v>
       </c>
       <c r="AK8" t="n">
-        <v>1.745635268477249</v>
+        <v>1.950891352838665</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.9354838709677419</v>
+        <v>0.9426229508196722</v>
       </c>
       <c r="AM8" t="n">
-        <v>214.728675813495</v>
+        <v>215.4492418397148</v>
       </c>
       <c r="AN8" t="n">
-        <v>530.0687403944672</v>
+        <v>531.8474945568648</v>
       </c>
       <c r="AO8" t="n">
-        <v>318.3695468950214</v>
+        <v>320.5963369295761</v>
       </c>
       <c r="AP8" t="n">
-        <v>233.5806631128492</v>
+        <v>233.5932123201758</v>
       </c>
       <c r="AQ8" t="n">
-        <v>403.1584306771937</v>
+        <v>407.5994615389765</v>
       </c>
       <c r="AR8" t="n">
-        <v>225.0507186256265</v>
+        <v>225.7991528435473</v>
       </c>
       <c r="AS8" t="n">
-        <v>439.3467810458824</v>
+        <v>445.6972459736809</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3338,19 +4697,19 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>385.73</v>
+        <v>396.6</v>
       </c>
       <c r="I9" t="n">
-        <v>6.02</v>
+        <v>6.03</v>
       </c>
       <c r="J9" t="n">
-        <v>64.07474999999999</v>
+        <v>65.77114</v>
       </c>
       <c r="K9" t="n">
         <v>33</v>
       </c>
       <c r="L9" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M9" t="n">
         <v>57.19493248774063</v>
@@ -3359,49 +4718,49 @@
         <v>93.87329577470153</v>
       </c>
       <c r="O9" t="n">
-        <v>74.91719886917585</v>
+        <v>75.04499179120712</v>
       </c>
       <c r="P9" t="n">
-        <v>78.39571411846676</v>
+        <v>78.71540210865163</v>
       </c>
       <c r="Q9" t="n">
-        <v>9.711013572373497</v>
+        <v>9.781241462981987</v>
       </c>
       <c r="R9" t="n">
-        <v>61.29707440530581</v>
+        <v>61.29473531920079</v>
       </c>
       <c r="S9" t="n">
-        <v>83.47290277016327</v>
+        <v>83.49376061274063</v>
       </c>
       <c r="T9" t="n">
-        <v>-1.116510525741735</v>
+        <v>-0.9481262502622875</v>
       </c>
       <c r="U9" t="n">
-        <v>0.253968253968254</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="V9" t="n">
-        <v>344.3134935761985</v>
+        <v>344.885442901076</v>
       </c>
       <c r="W9" t="n">
-        <v>565.1172405637031</v>
+        <v>566.0559735214503</v>
       </c>
       <c r="X9" t="n">
-        <v>451.0015371924386</v>
+        <v>452.521300500979</v>
       </c>
       <c r="Y9" t="n">
-        <v>392.5412354867501</v>
+        <v>393.5404144791976</v>
       </c>
       <c r="Z9" t="n">
-        <v>509.461838898127</v>
+        <v>511.5021865227603</v>
       </c>
       <c r="AA9" t="n">
-        <v>369.008387919941</v>
+        <v>369.6072539747808</v>
       </c>
       <c r="AB9" t="n">
-        <v>502.5068746763829</v>
+        <v>503.467376494826</v>
       </c>
       <c r="AC9" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AD9" t="n">
         <v>57.19493248774063</v>
@@ -3410,57 +4769,57 @@
         <v>93.87329577470153</v>
       </c>
       <c r="AF9" t="n">
-        <v>72.7265189141975</v>
+        <v>72.76569347655681</v>
       </c>
       <c r="AG9" t="n">
-        <v>71.83857403961119</v>
+        <v>71.85744439530923</v>
       </c>
       <c r="AH9" t="n">
-        <v>7.694561292849456</v>
+        <v>7.673032529667959</v>
       </c>
       <c r="AI9" t="n">
-        <v>62.49025281642149</v>
+        <v>62.51890781097711</v>
       </c>
       <c r="AJ9" t="n">
-        <v>82.3986358345136</v>
+        <v>82.39649127566095</v>
       </c>
       <c r="AK9" t="n">
-        <v>-1.124400545387504</v>
+        <v>-0.9115761531717999</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1709401709401709</v>
       </c>
       <c r="AM9" t="n">
-        <v>344.3134935761985</v>
+        <v>344.885442901076</v>
       </c>
       <c r="AN9" t="n">
-        <v>565.1172405637031</v>
+        <v>566.0559735214503</v>
       </c>
       <c r="AO9" t="n">
-        <v>437.8136438634689</v>
+        <v>438.7771316636375</v>
       </c>
       <c r="AP9" t="n">
-        <v>391.4923848805152</v>
+        <v>392.5087455097398</v>
       </c>
       <c r="AQ9" t="n">
-        <v>484.1349028464226</v>
+        <v>485.0455178175354</v>
       </c>
       <c r="AR9" t="n">
-        <v>376.1913219548574</v>
+        <v>376.989014100192</v>
       </c>
       <c r="AS9" t="n">
-        <v>496.0397877237718</v>
+        <v>496.8508423922356</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-06 01:09:28</t>
+          <t>2026-06-09 03:47:43</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3489,19 +4848,19 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>82.18000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I10" t="n">
         <v>3.1</v>
       </c>
       <c r="J10" t="n">
-        <v>26.509678</v>
+        <v>26.658066</v>
       </c>
       <c r="K10" t="n">
         <v>67</v>
       </c>
       <c r="L10" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="M10" t="n">
         <v>35.93675816954359</v>
@@ -3510,22 +4869,22 @@
         <v>42.60474344487245</v>
       </c>
       <c r="O10" t="n">
-        <v>38.41600789652239</v>
+        <v>38.40270594790844</v>
       </c>
       <c r="P10" t="n">
-        <v>37.71936770955563</v>
+        <v>37.65019654285294</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.917248392190739</v>
+        <v>1.990322096160243</v>
       </c>
       <c r="R10" t="n">
-        <v>36.41976247191899</v>
+        <v>36.38339890792905</v>
       </c>
       <c r="S10" t="n">
-        <v>41.14466490010498</v>
+        <v>41.39130483031742</v>
       </c>
       <c r="T10" t="n">
-        <v>-6.210113381770872</v>
+        <v>-5.900874019620422</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -3537,22 +4896,22 @@
         <v>132.0747046791046</v>
       </c>
       <c r="X10" t="n">
-        <v>119.0896244792194</v>
+        <v>119.0483884385162</v>
       </c>
       <c r="Y10" t="n">
-        <v>113.1461544634281</v>
+        <v>112.8783899404194</v>
       </c>
       <c r="Z10" t="n">
-        <v>125.0330944950107</v>
+        <v>125.2183869366129</v>
       </c>
       <c r="AA10" t="n">
-        <v>112.9012636629489</v>
+        <v>112.7885366145801</v>
       </c>
       <c r="AB10" t="n">
-        <v>127.5484611903254</v>
+        <v>128.313044973984</v>
       </c>
       <c r="AC10" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="AD10" t="n">
         <v>3.489557264641911</v>
@@ -3561,25 +4920,25 @@
         <v>42.60474344487245</v>
       </c>
       <c r="AF10" t="n">
-        <v>24.66089290957747</v>
+        <v>25.3821414425773</v>
       </c>
       <c r="AG10" t="n">
-        <v>32.4901173708467</v>
+        <v>32.59090830686063</v>
       </c>
       <c r="AH10" t="n">
-        <v>15.57837686140042</v>
+        <v>15.350467123509</v>
       </c>
       <c r="AI10" t="n">
-        <v>3.779782746967516</v>
+        <v>3.777151179492922</v>
       </c>
       <c r="AJ10" t="n">
-        <v>39.10988125405291</v>
+        <v>39.12055275656958</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.1186763619131203</v>
+        <v>0.08311959155097284</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.3483146067415731</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="AM10" t="n">
         <v>10.81762752038992</v>
@@ -3588,19 +4947,19 @@
         <v>132.0747046791046</v>
       </c>
       <c r="AO10" t="n">
-        <v>76.44876801969015</v>
+        <v>78.68463847198962</v>
       </c>
       <c r="AP10" t="n">
-        <v>28.15579974934885</v>
+        <v>31.09819038911171</v>
       </c>
       <c r="AQ10" t="n">
-        <v>124.7417362900314</v>
+        <v>126.2710865548675</v>
       </c>
       <c r="AR10" t="n">
-        <v>11.7173265155993</v>
+        <v>11.70916865642806</v>
       </c>
       <c r="AS10" t="n">
-        <v>121.240631887564</v>
+        <v>121.2737135453657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>